<commit_message>
Reverse epoch 2: her side veils on Changli's dress panels; pad texels below alpha 64
- The loose lilac strip at her hip was her SKIRT component's side veil (paint tests: not the
  sheer dress, not the shawl), its chain bones (240-242, 249-251) mapped onto Changli's coat
  sashes (258/259, 263/264), which swing free. They go to Changli's dress side-panel chain
  (92/93, 104/105) now -- the chain her sheer drapes already map onto -- in VGRemapData.cpp and
  in ChangliRemapDraft.xlsx's reverse sheet. In game the veils hang with the dress.
- The padding treats a texel below alpha 64 (three-quarters see-through on her own shader) as
  hidden, not only alpha 0: the back chains' grey was faint, not zero. They now draw as thin
  gold-brown cords; a fine cut-out chain cannot be drawn by an opaque shader, which
  remapGrading now says.

A/B byte-identical on all five skin mods.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Data/RemapDrafts/ChangliRemapDraft.xlsx
+++ b/Data/RemapDrafts/ChangliRemapDraft.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A5"/>
+  <dimension ref="A1:A4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -456,7 +456,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
@@ -471,7 +470,6 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A4" r:id="rId1"/>
@@ -8854,14 +8852,14 @@
         <v>240</v>
       </c>
       <c r="B242" t="n">
-        <v>259</v>
+        <v>92</v>
       </c>
       <c r="C242" t="n">
         <v>0.28</v>
       </c>
       <c r="D242" t="inlineStr">
         <is>
-          <t>260 verts (Component 5) -&gt; 155 verts (Component 5), dist 4.3168; runner-up 258 at dist 11.4962</t>
+          <t>IN-GAME AUDIT (reverse epoch 2, 2026-10-21): her side-veil chain goes to Changli's dress side-panel chain, not the coat sash it was mapped to (259), which swings free -- the veil peeled off her hip and hung in mid-air. [before: 260 verts (Component 5) -&gt; 155 verts (Component 5), dist 4.3168; runner-up 258 at dist 11.4962]</t>
         </is>
       </c>
     </row>
@@ -8870,14 +8868,14 @@
         <v>241</v>
       </c>
       <c r="B243" t="n">
-        <v>258</v>
+        <v>93</v>
       </c>
       <c r="C243" t="n">
         <v>0.722</v>
       </c>
       <c r="D243" t="inlineStr">
         <is>
-          <t>204 verts (Component 5) -&gt; 158 verts (Component 5), dist 8.4340; runner-up 259 at dist 9.6326</t>
+          <t>IN-GAME AUDIT (reverse epoch 2, 2026-10-21): her side-veil chain goes to Changli's dress side-panel chain, not the coat sash it was mapped to (258), which swings free -- the veil peeled off her hip and hung in mid-air. [before: 204 verts (Component 5) -&gt; 158 verts (Component 5), dist 8.4340; runner-up 259 at dist 9.6326]</t>
         </is>
       </c>
     </row>
@@ -8886,14 +8884,14 @@
         <v>242</v>
       </c>
       <c r="B244" t="n">
-        <v>258</v>
+        <v>93</v>
       </c>
       <c r="C244" t="n">
         <v>0.976</v>
       </c>
       <c r="D244" t="inlineStr">
         <is>
-          <t>124 verts (Component 5) -&gt; 158 verts (Component 5), dist 9.4179; runner-up 259 at dist 13.1920</t>
+          <t>IN-GAME AUDIT (reverse epoch 2, 2026-10-21): her side-veil chain goes to Changli's dress side-panel chain, not the coat sash it was mapped to (258), which swings free -- the veil peeled off her hip and hung in mid-air. [before: 124 verts (Component 5) -&gt; 158 verts (Component 5), dist 9.4179; runner-up 259 at dist 13.1920]</t>
         </is>
       </c>
     </row>
@@ -8998,14 +8996,14 @@
         <v>249</v>
       </c>
       <c r="B251" t="n">
-        <v>264</v>
+        <v>104</v>
       </c>
       <c r="C251" t="n">
         <v>0.28</v>
       </c>
       <c r="D251" t="inlineStr">
         <is>
-          <t>260 verts (Component 5) -&gt; 155 verts (Component 5), dist 4.3168; runner-up 263 at dist 11.4962</t>
+          <t>IN-GAME AUDIT (reverse epoch 2, 2026-10-21): her side-veil chain goes to Changli's dress side-panel chain, not the coat sash it was mapped to (264), which swings free -- the veil peeled off her hip and hung in mid-air. [before: 260 verts (Component 5) -&gt; 155 verts (Component 5), dist 4.3168; runner-up 263 at dist 11.4962]</t>
         </is>
       </c>
     </row>
@@ -9014,14 +9012,14 @@
         <v>250</v>
       </c>
       <c r="B252" t="n">
-        <v>263</v>
+        <v>105</v>
       </c>
       <c r="C252" t="n">
         <v>0.722</v>
       </c>
       <c r="D252" t="inlineStr">
         <is>
-          <t>204 verts (Component 5) -&gt; 158 verts (Component 5), dist 8.4340; runner-up 264 at dist 9.6326</t>
+          <t>IN-GAME AUDIT (reverse epoch 2, 2026-10-21): her side-veil chain goes to Changli's dress side-panel chain, not the coat sash it was mapped to (263), which swings free -- the veil peeled off her hip and hung in mid-air. [before: 204 verts (Component 5) -&gt; 158 verts (Component 5), dist 8.4340; runner-up 264 at dist 9.6326]</t>
         </is>
       </c>
     </row>
@@ -9030,14 +9028,14 @@
         <v>251</v>
       </c>
       <c r="B253" t="n">
-        <v>263</v>
+        <v>105</v>
       </c>
       <c r="C253" t="n">
         <v>0.976</v>
       </c>
       <c r="D253" t="inlineStr">
         <is>
-          <t>124 verts (Component 5) -&gt; 158 verts (Component 5), dist 9.4179; runner-up 264 at dist 13.1920</t>
+          <t>IN-GAME AUDIT (reverse epoch 2, 2026-10-21): her side-veil chain goes to Changli's dress side-panel chain, not the coat sash it was mapped to (263), which swings free -- the veil peeled off her hip and hung in mid-air. [before: 124 verts (Component 5) -&gt; 158 verts (Component 5), dist 9.4179; runner-up 264 at dist 13.1920]</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Reverse epoch 3: her right side veil on Changli's right thigh
Changli's right dress panel (92 / 93, the buckle side) is turned in her
idle, so the veil remapped onto it hung edge-on. The three right-veil
bones (240-242) go to the rigid right thigh (173) now; the left veil stays
on the left panel. Checked in game on the identity mod; the prototype and
the compiled fix are identical on all five skin mods.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Data/RemapDrafts/ChangliRemapDraft.xlsx
+++ b/Data/RemapDrafts/ChangliRemapDraft.xlsx
@@ -8852,14 +8852,14 @@
         <v>240</v>
       </c>
       <c r="B242" t="n">
-        <v>92</v>
+        <v>173</v>
       </c>
       <c r="C242" t="n">
         <v>0.28</v>
       </c>
       <c r="D242" t="inlineStr">
         <is>
-          <t>IN-GAME AUDIT (reverse epoch 2, 2026-10-21): her side-veil chain goes to Changli's dress side-panel chain, not the coat sash it was mapped to (259), which swings free -- the veil peeled off her hip and hung in mid-air. [before: 260 verts (Component 5) -&gt; 155 verts (Component 5), dist 4.3168; runner-up 258 at dist 11.4962]</t>
+          <t>IN-GAME AUDIT (reverse epoch 3, 2026-10-21): the right side veil goes to Changli's right thigh (173), a rigid leg bone: her right dress panel (92 / 93, the buckle side) is turned in her idle and the veil hung edge-on on it (epoch 3; before that, 92). IN-GAME AUDIT (reverse epoch 2, 2026-10-21): her side-veil chain goes to Changli's dress side-panel chain, not the coat sash it was mapped to (259), which swings free -- the veil peeled off her hip and hung in mid-air. [before: 260 verts (Component 5) -&gt; 155 verts (Component 5), dist 4.3168; runner-up 258 at dist 11.4962]</t>
         </is>
       </c>
     </row>
@@ -8868,14 +8868,14 @@
         <v>241</v>
       </c>
       <c r="B243" t="n">
-        <v>93</v>
+        <v>173</v>
       </c>
       <c r="C243" t="n">
         <v>0.722</v>
       </c>
       <c r="D243" t="inlineStr">
         <is>
-          <t>IN-GAME AUDIT (reverse epoch 2, 2026-10-21): her side-veil chain goes to Changli's dress side-panel chain, not the coat sash it was mapped to (258), which swings free -- the veil peeled off her hip and hung in mid-air. [before: 204 verts (Component 5) -&gt; 158 verts (Component 5), dist 8.4340; runner-up 259 at dist 9.6326]</t>
+          <t>IN-GAME AUDIT (reverse epoch 3, 2026-10-21): the right side veil goes to Changli's right thigh (173), a rigid leg bone: her right dress panel (92 / 93, the buckle side) is turned in her idle and the veil hung edge-on on it (epoch 3; before that, 93). IN-GAME AUDIT (reverse epoch 2, 2026-10-21): her side-veil chain goes to Changli's dress side-panel chain, not the coat sash it was mapped to (258), which swings free -- the veil peeled off her hip and hung in mid-air. [before: 204 verts (Component 5) -&gt; 158 verts (Component 5), dist 8.4340; runner-up 259 at dist 9.6326]</t>
         </is>
       </c>
     </row>
@@ -8884,14 +8884,14 @@
         <v>242</v>
       </c>
       <c r="B244" t="n">
-        <v>93</v>
+        <v>173</v>
       </c>
       <c r="C244" t="n">
         <v>0.976</v>
       </c>
       <c r="D244" t="inlineStr">
         <is>
-          <t>IN-GAME AUDIT (reverse epoch 2, 2026-10-21): her side-veil chain goes to Changli's dress side-panel chain, not the coat sash it was mapped to (258), which swings free -- the veil peeled off her hip and hung in mid-air. [before: 124 verts (Component 5) -&gt; 158 verts (Component 5), dist 9.4179; runner-up 259 at dist 13.1920]</t>
+          <t>IN-GAME AUDIT (reverse epoch 3, 2026-10-21): the right side veil goes to Changli's right thigh (173), a rigid leg bone: her right dress panel (92 / 93, the buckle side) is turned in her idle and the veil hung edge-on on it (epoch 3; before that, 93). IN-GAME AUDIT (reverse epoch 2, 2026-10-21): her side-veil chain goes to Changli's dress side-panel chain, not the coat sash it was mapped to (258), which swings free -- the veil peeled off her hip and hung in mid-air. [before: 124 verts (Component 5) -&gt; 158 verts (Component 5), dist 9.4179; runner-up 259 at dist 13.1920]</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Reverse epoch 4: her right side veil back on Changli's right panel
Epochs 3 and 4 saw the skin's right side panel edge-on from straight in
front, on Changli's right panel, her right thigh and her pelvis alike. The
panels are modelled facing sideways (normal along x, 24.5 units deep), and
the skin's own idle swings the right one round to face front; Changli's
does not. That is the pose, not the row, so the right veil goes back to
the mirror of the left (92 / 93), byte-identical to the epoch-3 build.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Data/RemapDrafts/ChangliRemapDraft.xlsx
+++ b/Data/RemapDrafts/ChangliRemapDraft.xlsx
@@ -8852,14 +8852,14 @@
         <v>240</v>
       </c>
       <c r="B242" t="n">
-        <v>173</v>
+        <v>92</v>
       </c>
       <c r="C242" t="n">
         <v>0.28</v>
       </c>
       <c r="D242" t="inlineStr">
         <is>
-          <t>IN-GAME AUDIT (reverse epoch 3, 2026-10-21): the right side veil goes to Changli's right thigh (173), a rigid leg bone: her right dress panel (92 / 93, the buckle side) is turned in her idle and the veil hung edge-on on it (epoch 3; before that, 92). IN-GAME AUDIT (reverse epoch 2, 2026-10-21): her side-veil chain goes to Changli's dress side-panel chain, not the coat sash it was mapped to (259), which swings free -- the veil peeled off her hip and hung in mid-air. [before: 260 verts (Component 5) -&gt; 155 verts (Component 5), dist 4.3168; runner-up 258 at dist 11.4962]</t>
+          <t>IN-GAME AUDIT (reverse epochs 3-4, 2026-10-21): kept on Changli's right dress side panel, the mirror of the left veil. Seen from straight in front her right side panel is edge-on on Changli and broad on the skin's card: both panels are modelled facing sideways and the skin's idle turns the right one to the front. Her right thigh (173) and pelvis (170) left it edge-on just the same. IN-GAME AUDIT (reverse epoch 2, 2026-10-21): her side-veil chain goes to Changli's dress side-panel chain, not the coat sash it was mapped to (259), which swings free -- the veil peeled off her hip and hung in mid-air. [before: 260 verts (Component 5) -&gt; 155 verts (Component 5), dist 4.3168; runner-up 258 at dist 11.4962]</t>
         </is>
       </c>
     </row>
@@ -8868,14 +8868,14 @@
         <v>241</v>
       </c>
       <c r="B243" t="n">
-        <v>173</v>
+        <v>93</v>
       </c>
       <c r="C243" t="n">
         <v>0.722</v>
       </c>
       <c r="D243" t="inlineStr">
         <is>
-          <t>IN-GAME AUDIT (reverse epoch 3, 2026-10-21): the right side veil goes to Changli's right thigh (173), a rigid leg bone: her right dress panel (92 / 93, the buckle side) is turned in her idle and the veil hung edge-on on it (epoch 3; before that, 93). IN-GAME AUDIT (reverse epoch 2, 2026-10-21): her side-veil chain goes to Changli's dress side-panel chain, not the coat sash it was mapped to (258), which swings free -- the veil peeled off her hip and hung in mid-air. [before: 204 verts (Component 5) -&gt; 158 verts (Component 5), dist 8.4340; runner-up 259 at dist 9.6326]</t>
+          <t>IN-GAME AUDIT (reverse epochs 3-4, 2026-10-21): kept on Changli's right dress side panel, the mirror of the left veil. Seen from straight in front her right side panel is edge-on on Changli and broad on the skin's card: both panels are modelled facing sideways and the skin's idle turns the right one to the front. Her right thigh (173) and pelvis (170) left it edge-on just the same. IN-GAME AUDIT (reverse epoch 2, 2026-10-21): her side-veil chain goes to Changli's dress side-panel chain, not the coat sash it was mapped to (258), which swings free -- the veil peeled off her hip and hung in mid-air. [before: 204 verts (Component 5) -&gt; 158 verts (Component 5), dist 8.4340; runner-up 259 at dist 9.6326]</t>
         </is>
       </c>
     </row>
@@ -8884,14 +8884,14 @@
         <v>242</v>
       </c>
       <c r="B244" t="n">
-        <v>173</v>
+        <v>93</v>
       </c>
       <c r="C244" t="n">
         <v>0.976</v>
       </c>
       <c r="D244" t="inlineStr">
         <is>
-          <t>IN-GAME AUDIT (reverse epoch 3, 2026-10-21): the right side veil goes to Changli's right thigh (173), a rigid leg bone: her right dress panel (92 / 93, the buckle side) is turned in her idle and the veil hung edge-on on it (epoch 3; before that, 93). IN-GAME AUDIT (reverse epoch 2, 2026-10-21): her side-veil chain goes to Changli's dress side-panel chain, not the coat sash it was mapped to (258), which swings free -- the veil peeled off her hip and hung in mid-air. [before: 124 verts (Component 5) -&gt; 158 verts (Component 5), dist 9.4179; runner-up 259 at dist 13.1920]</t>
+          <t>IN-GAME AUDIT (reverse epochs 3-4, 2026-10-21): kept on Changli's right dress side panel, the mirror of the left veil. Seen from straight in front her right side panel is edge-on on Changli and broad on the skin's card: both panels are modelled facing sideways and the skin's idle turns the right one to the front. Her right thigh (173) and pelvis (170) left it edge-on just the same. IN-GAME AUDIT (reverse epoch 2, 2026-10-21): her side-veil chain goes to Changli's dress side-panel chain, not the coat sash it was mapped to (258), which swings free -- the veil peeled off her hip and hung in mid-air. [before: 124 verts (Component 5) -&gt; 158 verts (Component 5), dist 9.4179; runner-up 259 at dist 13.1920]</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Join The Council: The Borrowed Shader Smith (68)
Carried each character's own game shaders onto the other for Changli <-> ChangliNymph,
and made them fade with the body. Both counters 67 -> 68 (the roster sums to 68), and a
credit row in ChangliRemapDraft.xlsx.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Data/RemapDrafts/ChangliRemapDraft.xlsx
+++ b/Data/RemapDrafts/ChangliRemapDraft.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A4"/>
+  <dimension ref="A1:A5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -470,9 +470,17 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>🔥🎭 The Borrowed Shader Smith: The 68th member of The Council</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A4" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>